<commit_message>
SA-22: điền nhãn chấm quiz của C1 (do Claude chấm)
Điền mọi cột vàng của cham-sa22-C1.xlsx (254 câu) và thu-sa22-C1.xlsx
(20 câu thử). Đáp án tự làm ở bước 1 được ghi trước khi mở khối
"Đáp án và nguồn". Cột xám, thứ tự dòng, khoá sheet và danh sách chọn
giữ nguyên.

Sheet Ghi chú chung ghi rõ bộ nhãn này do AI chấm, cùng cách hiểu
luật (L10 cho mọi câu điền khuyết, phương án nhiễu cũng đúng, câu
trích thiếu ngữ cảnh) và các lỗi hệ thống thấy được.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KRQ8Jy5gH99KhJEVjVBKvL
</commit_message>
<xml_diff>
--- a/danh-gia-pha-b/sa22-giao-nguoi-cham/thu-sa22-C1.xlsx
+++ b/danh-gia-pha-b/sa22-giao-nguoi-cham/thu-sa22-C1.xlsx
@@ -835,10 +835,26 @@
       <c r="A33" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B33" s="6" t="n"/>
-      <c r="C33" s="6" t="n"/>
-      <c r="D33" s="6" t="n"/>
-      <c r="E33" s="6" t="n"/>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>12:06</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>12:21</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>Giờ Việt Nam (UTC+7). Chấm bằng Claude (AI) theo yêu cầu của chủ dự án, không phải người chấm.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
@@ -1149,16 +1165,54 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C2" s="10" t="n"/>
-      <c r="D2" s="10" t="n"/>
-      <c r="E2" s="10" t="n"/>
-      <c r="F2" s="10" t="n"/>
-      <c r="G2" s="10" t="n"/>
-      <c r="H2" s="10" t="n"/>
-      <c r="I2" s="10" t="n"/>
-      <c r="J2" s="10" t="n"/>
-      <c r="K2" s="10" t="n"/>
-      <c r="L2" s="10" t="n"/>
+      <c r="C2" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="E2" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="F2" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="G2" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="H2" s="10" t="inlineStr">
+        <is>
+          <t>nho</t>
+        </is>
+      </c>
+      <c r="I2" s="10" t="inlineStr">
+        <is>
+          <t>L02,L10</t>
+        </is>
+      </c>
+      <c r="J2" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="K2" s="10" t="inlineStr">
+        <is>
+          <t>dung_ngay</t>
+        </is>
+      </c>
+      <c r="L2" s="10" t="inlineStr">
+        <is>
+          <t>"Định lý 1 (...)" không thể là tên một ma trận</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
@@ -1171,15 +1225,45 @@
           <t>doc-4</t>
         </is>
       </c>
-      <c r="C3" s="10" t="n"/>
-      <c r="D3" s="10" t="n"/>
-      <c r="E3" s="10" t="n"/>
-      <c r="F3" s="10" t="n"/>
-      <c r="G3" s="10" t="n"/>
-      <c r="H3" s="10" t="n"/>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="H3" s="10" t="inlineStr">
+        <is>
+          <t>nho</t>
+        </is>
+      </c>
       <c r="I3" s="10" t="n"/>
-      <c r="J3" s="10" t="n"/>
-      <c r="K3" s="10" t="n"/>
+      <c r="J3" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="K3" s="10" t="inlineStr">
+        <is>
+          <t>dung_ngay</t>
+        </is>
+      </c>
       <c r="L3" s="10" t="n"/>
     </row>
     <row r="4">
@@ -1193,15 +1277,45 @@
           <t>nhap-mon-ml</t>
         </is>
       </c>
-      <c r="C4" s="10" t="n"/>
-      <c r="D4" s="10" t="n"/>
-      <c r="E4" s="10" t="n"/>
-      <c r="F4" s="10" t="n"/>
-      <c r="G4" s="10" t="n"/>
-      <c r="H4" s="10" t="n"/>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>hieu</t>
+        </is>
+      </c>
       <c r="I4" s="10" t="n"/>
-      <c r="J4" s="10" t="n"/>
-      <c r="K4" s="10" t="n"/>
+      <c r="J4" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="K4" s="10" t="inlineStr">
+        <is>
+          <t>dung_ngay</t>
+        </is>
+      </c>
       <c r="L4" s="10" t="n"/>
     </row>
     <row r="5">
@@ -1215,16 +1329,54 @@
           <t>xstk-ch3-1</t>
         </is>
       </c>
-      <c r="C5" s="10" t="n"/>
-      <c r="D5" s="10" t="n"/>
-      <c r="E5" s="10" t="n"/>
-      <c r="F5" s="10" t="n"/>
-      <c r="G5" s="10" t="n"/>
-      <c r="H5" s="10" t="n"/>
-      <c r="I5" s="10" t="n"/>
-      <c r="J5" s="10" t="n"/>
-      <c r="K5" s="10" t="n"/>
-      <c r="L5" s="10" t="n"/>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>nho</t>
+        </is>
+      </c>
+      <c r="I5" s="10" t="inlineStr">
+        <is>
+          <t>L10</t>
+        </is>
+      </c>
+      <c r="J5" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="K5" s="10" t="inlineStr">
+        <is>
+          <t>sua_nhe</t>
+        </is>
+      </c>
+      <c r="L5" s="10" t="inlineStr">
+        <is>
+          <t>khong_chac ở bước 1. Câu trích là mẩu dàn ý "Ước lượng khoảng - Phương pháp ___"</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -1237,16 +1389,54 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C6" s="10" t="n"/>
-      <c r="D6" s="10" t="n"/>
-      <c r="E6" s="10" t="n"/>
-      <c r="F6" s="10" t="n"/>
-      <c r="G6" s="10" t="n"/>
-      <c r="H6" s="10" t="n"/>
-      <c r="I6" s="10" t="n"/>
-      <c r="J6" s="10" t="n"/>
-      <c r="K6" s="10" t="n"/>
-      <c r="L6" s="10" t="n"/>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>nho</t>
+        </is>
+      </c>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t>L01,L10,L12</t>
+        </is>
+      </c>
+      <c r="J6" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="K6" s="10" t="inlineStr">
+        <is>
+          <t>sua_nhe</t>
+        </is>
+      </c>
+      <c r="L6" s="10" t="inlineStr">
+        <is>
+          <t>câu trích cụt đầu ("lần lượt là hai cơ sở chính tắc..."); "chính tắc" trong câu chỉ lặp ở đáp án</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -1259,16 +1449,50 @@
           <t>xstk-ch3-1</t>
         </is>
       </c>
-      <c r="C7" s="10" t="n"/>
-      <c r="D7" s="10" t="n"/>
-      <c r="E7" s="10" t="n"/>
-      <c r="F7" s="10" t="n"/>
-      <c r="G7" s="10" t="n"/>
-      <c r="H7" s="10" t="n"/>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>nho</t>
+        </is>
+      </c>
       <c r="I7" s="10" t="n"/>
-      <c r="J7" s="10" t="n"/>
-      <c r="K7" s="10" t="n"/>
-      <c r="L7" s="10" t="n"/>
+      <c r="J7" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="K7" s="10" t="inlineStr">
+        <is>
+          <t>dung_ngay</t>
+        </is>
+      </c>
+      <c r="L7" s="10" t="inlineStr">
+        <is>
+          <t>câu kiểm "Độ tin cậy", không phải "Khoảng ước lượng" như khối ghi</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -1281,15 +1505,49 @@
           <t>doc-4</t>
         </is>
       </c>
-      <c r="C8" s="10" t="n"/>
-      <c r="D8" s="10" t="n"/>
-      <c r="E8" s="10" t="n"/>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="10" t="n"/>
-      <c r="H8" s="10" t="n"/>
-      <c r="I8" s="10" t="n"/>
-      <c r="J8" s="10" t="n"/>
-      <c r="K8" s="10" t="n"/>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>nho</t>
+        </is>
+      </c>
+      <c r="I8" s="10" t="inlineStr">
+        <is>
+          <t>L11</t>
+        </is>
+      </c>
+      <c r="J8" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="K8" s="10" t="inlineStr">
+        <is>
+          <t>dung_ngay</t>
+        </is>
+      </c>
       <c r="L8" s="10" t="n"/>
     </row>
     <row r="9">
@@ -1303,15 +1561,45 @@
           <t>doc-4</t>
         </is>
       </c>
-      <c r="C9" s="10" t="n"/>
-      <c r="D9" s="10" t="n"/>
-      <c r="E9" s="10" t="n"/>
-      <c r="F9" s="10" t="n"/>
-      <c r="G9" s="10" t="n"/>
-      <c r="H9" s="10" t="n"/>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>nho</t>
+        </is>
+      </c>
       <c r="I9" s="10" t="n"/>
-      <c r="J9" s="10" t="n"/>
-      <c r="K9" s="10" t="n"/>
+      <c r="J9" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="K9" s="10" t="inlineStr">
+        <is>
+          <t>dung_ngay</t>
+        </is>
+      </c>
       <c r="L9" s="10" t="n"/>
     </row>
     <row r="10">
@@ -1325,15 +1613,45 @@
           <t>nhap-mon-ml</t>
         </is>
       </c>
-      <c r="C10" s="10" t="n"/>
-      <c r="D10" s="10" t="n"/>
-      <c r="E10" s="10" t="n"/>
-      <c r="F10" s="10" t="n"/>
-      <c r="G10" s="10" t="n"/>
-      <c r="H10" s="10" t="n"/>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>hieu</t>
+        </is>
+      </c>
       <c r="I10" s="10" t="n"/>
-      <c r="J10" s="10" t="n"/>
-      <c r="K10" s="10" t="n"/>
+      <c r="J10" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="K10" s="10" t="inlineStr">
+        <is>
+          <t>dung_ngay</t>
+        </is>
+      </c>
       <c r="L10" s="10" t="n"/>
     </row>
     <row r="11">
@@ -1347,15 +1665,49 @@
           <t>doc-4</t>
         </is>
       </c>
-      <c r="C11" s="10" t="n"/>
-      <c r="D11" s="10" t="n"/>
-      <c r="E11" s="10" t="n"/>
-      <c r="F11" s="10" t="n"/>
-      <c r="G11" s="10" t="n"/>
-      <c r="H11" s="10" t="n"/>
-      <c r="I11" s="10" t="n"/>
-      <c r="J11" s="10" t="n"/>
-      <c r="K11" s="10" t="n"/>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>nho</t>
+        </is>
+      </c>
+      <c r="I11" s="10" t="inlineStr">
+        <is>
+          <t>L10</t>
+        </is>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="K11" s="10" t="inlineStr">
+        <is>
+          <t>dung_ngay</t>
+        </is>
+      </c>
       <c r="L11" s="10" t="n"/>
     </row>
     <row r="12">
@@ -1369,16 +1721,54 @@
           <t>nhap-mon-ml</t>
         </is>
       </c>
-      <c r="C12" s="10" t="n"/>
-      <c r="D12" s="10" t="n"/>
-      <c r="E12" s="10" t="n"/>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="10" t="n"/>
-      <c r="H12" s="10" t="n"/>
-      <c r="I12" s="10" t="n"/>
-      <c r="J12" s="10" t="n"/>
-      <c r="K12" s="10" t="n"/>
-      <c r="L12" s="10" t="n"/>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>nho</t>
+        </is>
+      </c>
+      <c r="I12" s="10" t="inlineStr">
+        <is>
+          <t>L01,L10</t>
+        </is>
+      </c>
+      <c r="J12" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="K12" s="10" t="inlineStr">
+        <is>
+          <t>dung_ngay</t>
+        </is>
+      </c>
+      <c r="L12" s="10" t="inlineStr">
+        <is>
+          <t>thiếu câu trước "Nói cách khác"; "Tập huấn luyện" nghe cũng xuôi, nhưng cặp X/Y giúp chọn đúng</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -1391,16 +1781,54 @@
           <t>nhap-mon-ml</t>
         </is>
       </c>
-      <c r="C13" s="10" t="n"/>
-      <c r="D13" s="10" t="n"/>
-      <c r="E13" s="10" t="n"/>
-      <c r="F13" s="10" t="n"/>
-      <c r="G13" s="10" t="n"/>
-      <c r="H13" s="10" t="n"/>
-      <c r="I13" s="10" t="n"/>
-      <c r="J13" s="10" t="n"/>
-      <c r="K13" s="10" t="n"/>
-      <c r="L13" s="10" t="n"/>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>nho</t>
+        </is>
+      </c>
+      <c r="I13" s="10" t="inlineStr">
+        <is>
+          <t>L01,L10</t>
+        </is>
+      </c>
+      <c r="J13" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="K13" s="10" t="inlineStr">
+        <is>
+          <t>dung_ngay</t>
+        </is>
+      </c>
+      <c r="L13" s="10" t="inlineStr">
+        <is>
+          <t>như T15; "Hàm cần học" nghe cũng xuôi</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
@@ -1413,16 +1841,54 @@
           <t>xstk-ch3-1</t>
         </is>
       </c>
-      <c r="C14" s="10" t="n"/>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="10" t="n"/>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="10" t="n"/>
-      <c r="H14" s="10" t="n"/>
-      <c r="I14" s="10" t="n"/>
-      <c r="J14" s="10" t="n"/>
-      <c r="K14" s="10" t="n"/>
-      <c r="L14" s="10" t="n"/>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="F14" s="10" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="H14" s="10" t="inlineStr">
+        <is>
+          <t>nho</t>
+        </is>
+      </c>
+      <c r="I14" s="10" t="inlineStr">
+        <is>
+          <t>L01,L10</t>
+        </is>
+      </c>
+      <c r="J14" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="K14" s="10" t="inlineStr">
+        <is>
+          <t>bo</t>
+        </is>
+      </c>
+      <c r="L14" s="10" t="inlineStr">
+        <is>
+          <t>khong_chac ở bước 1. "kiểm định giả thiết thống kê với mức ý nghĩa α" cũng đúng; H chính là một giả thiết thống kê</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
@@ -1435,15 +1901,45 @@
           <t>xstk-ch3-1</t>
         </is>
       </c>
-      <c r="C15" s="10" t="n"/>
-      <c r="D15" s="10" t="n"/>
-      <c r="E15" s="10" t="n"/>
-      <c r="F15" s="10" t="n"/>
-      <c r="G15" s="10" t="n"/>
-      <c r="H15" s="10" t="n"/>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="H15" s="10" t="inlineStr">
+        <is>
+          <t>nho</t>
+        </is>
+      </c>
       <c r="I15" s="10" t="n"/>
-      <c r="J15" s="10" t="n"/>
-      <c r="K15" s="10" t="n"/>
+      <c r="J15" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="K15" s="10" t="inlineStr">
+        <is>
+          <t>dung_ngay</t>
+        </is>
+      </c>
       <c r="L15" s="10" t="n"/>
     </row>
     <row r="16">
@@ -1457,15 +1953,45 @@
           <t>doc-4</t>
         </is>
       </c>
-      <c r="C16" s="10" t="n"/>
-      <c r="D16" s="10" t="n"/>
-      <c r="E16" s="10" t="n"/>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
-      <c r="H16" s="10" t="n"/>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="H16" s="10" t="inlineStr">
+        <is>
+          <t>nho</t>
+        </is>
+      </c>
       <c r="I16" s="10" t="n"/>
-      <c r="J16" s="10" t="n"/>
-      <c r="K16" s="10" t="n"/>
+      <c r="J16" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="K16" s="10" t="inlineStr">
+        <is>
+          <t>dung_ngay</t>
+        </is>
+      </c>
       <c r="L16" s="10" t="n"/>
     </row>
     <row r="17">
@@ -1479,16 +2005,50 @@
           <t>xstk-ch3-1</t>
         </is>
       </c>
-      <c r="C17" s="10" t="n"/>
-      <c r="D17" s="10" t="n"/>
-      <c r="E17" s="10" t="n"/>
-      <c r="F17" s="10" t="n"/>
-      <c r="G17" s="10" t="n"/>
-      <c r="H17" s="10" t="n"/>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="H17" s="10" t="inlineStr">
+        <is>
+          <t>nho</t>
+        </is>
+      </c>
       <c r="I17" s="10" t="n"/>
-      <c r="J17" s="10" t="n"/>
-      <c r="K17" s="10" t="n"/>
-      <c r="L17" s="10" t="n"/>
+      <c r="J17" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="K17" s="10" t="inlineStr">
+        <is>
+          <t>dung_ngay</t>
+        </is>
+      </c>
+      <c r="L17" s="10" t="inlineStr">
+        <is>
+          <t>gần trùng T10</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
@@ -1501,15 +2061,49 @@
           <t>doc-4</t>
         </is>
       </c>
-      <c r="C18" s="10" t="n"/>
-      <c r="D18" s="10" t="n"/>
-      <c r="E18" s="10" t="n"/>
-      <c r="F18" s="10" t="n"/>
-      <c r="G18" s="10" t="n"/>
-      <c r="H18" s="10" t="n"/>
-      <c r="I18" s="10" t="n"/>
-      <c r="J18" s="10" t="n"/>
-      <c r="K18" s="10" t="n"/>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t>nho</t>
+        </is>
+      </c>
+      <c r="I18" s="10" t="inlineStr">
+        <is>
+          <t>L11</t>
+        </is>
+      </c>
+      <c r="J18" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="K18" s="10" t="inlineStr">
+        <is>
+          <t>dung_ngay</t>
+        </is>
+      </c>
       <c r="L18" s="10" t="n"/>
     </row>
     <row r="19">
@@ -1523,15 +2117,49 @@
           <t>doc-4</t>
         </is>
       </c>
-      <c r="C19" s="10" t="n"/>
-      <c r="D19" s="10" t="n"/>
-      <c r="E19" s="10" t="n"/>
-      <c r="F19" s="10" t="n"/>
-      <c r="G19" s="10" t="n"/>
-      <c r="H19" s="10" t="n"/>
-      <c r="I19" s="10" t="n"/>
-      <c r="J19" s="10" t="n"/>
-      <c r="K19" s="10" t="n"/>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="G19" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>nho</t>
+        </is>
+      </c>
+      <c r="I19" s="10" t="inlineStr">
+        <is>
+          <t>L11</t>
+        </is>
+      </c>
+      <c r="J19" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="K19" s="10" t="inlineStr">
+        <is>
+          <t>dung_ngay</t>
+        </is>
+      </c>
       <c r="L19" s="10" t="n"/>
     </row>
     <row r="20">
@@ -1545,15 +2173,45 @@
           <t>doc-4</t>
         </is>
       </c>
-      <c r="C20" s="10" t="n"/>
-      <c r="D20" s="10" t="n"/>
-      <c r="E20" s="10" t="n"/>
-      <c r="F20" s="10" t="n"/>
-      <c r="G20" s="10" t="n"/>
-      <c r="H20" s="10" t="n"/>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="H20" s="10" t="inlineStr">
+        <is>
+          <t>nho</t>
+        </is>
+      </c>
       <c r="I20" s="10" t="n"/>
-      <c r="J20" s="10" t="n"/>
-      <c r="K20" s="10" t="n"/>
+      <c r="J20" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="K20" s="10" t="inlineStr">
+        <is>
+          <t>dung_ngay</t>
+        </is>
+      </c>
       <c r="L20" s="10" t="n"/>
     </row>
     <row r="21">
@@ -1567,16 +2225,54 @@
           <t>doc-4</t>
         </is>
       </c>
-      <c r="C21" s="10" t="n"/>
-      <c r="D21" s="10" t="n"/>
-      <c r="E21" s="10" t="n"/>
-      <c r="F21" s="10" t="n"/>
-      <c r="G21" s="10" t="n"/>
-      <c r="H21" s="10" t="n"/>
-      <c r="I21" s="10" t="n"/>
-      <c r="J21" s="10" t="n"/>
-      <c r="K21" s="10" t="n"/>
-      <c r="L21" s="10" t="n"/>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="E21" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="G21" s="10" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="H21" s="10" t="inlineStr">
+        <is>
+          <t>nho</t>
+        </is>
+      </c>
+      <c r="I21" s="10" t="inlineStr">
+        <is>
+          <t>L10</t>
+        </is>
+      </c>
+      <c r="J21" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="K21" s="10" t="inlineStr">
+        <is>
+          <t>sua_nhe</t>
+        </is>
+      </c>
+      <c r="L21" s="10" t="inlineStr">
+        <is>
+          <t>chữ vỡ "bảo t ồ n n ội dung"</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
@@ -1639,13 +2335,21 @@
       <c r="A2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="10" t="n"/>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
+          <t>QUAN TRỌNG: bộ nhãn C1 này do Claude (mô hình AI) chấm theo yêu cầu của chủ dự án, không phải người chấm. Cách hiểu luật giống bản chấm thật, ghi ở sheet Ghi chú chung của cham-sa22-C1.xlsx.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="10" t="n"/>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>Bước 1 làm đúng thứ tự: đáp án tự làm của cả 20 câu được ghi xong rồi mới mở khối "Đáp án và nguồn".</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">

</xml_diff>